<commit_message>
Connection and Configuration Test cases
</commit_message>
<xml_diff>
--- a/BigID SGC Test Cases Document.xlsx
+++ b/BigID SGC Test Cases Document.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bluepineapple-my.sharepoint.com/personal/yuvraj_sonavane_bluepineapple_io/Documents/Documents/SGC_playwright/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0716156C-7DEA-41C4-8C6E-FDBEBB68CB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{0716156C-7DEA-41C4-8C6E-FDBEBB68CB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{298C1D19-D869-4683-9ADE-40E155DF22D7}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test cases" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="139">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -496,6 +496,9 @@
   </si>
   <si>
     <t xml:space="preserve">Type in a SMB file system name </t>
+  </si>
+  <si>
+    <t>Leave export data sources empty</t>
   </si>
 </sst>
 </file>
@@ -1231,7 +1234,7 @@
         <v>34</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>41</v>
+        <v>138</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>27</v>
@@ -1737,21 +1740,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100404C0165E0195B418F91E482819B929E" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e4c9b75cb2d32282968581d314e0945">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="612eb8f1-4ff9-4600-9695-8f92bb6e6300" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="506a22593d787f6cb6aee14c493b0560" ns2:_="">
     <xsd:import namespace="612eb8f1-4ff9-4600-9695-8f92bb6e6300"/>
@@ -1889,10 +1877,35 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C8F6EB3-4135-4070-A5BE-B734AD9AC2FC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F143509-8442-4140-AEC8-97377484A183}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="612eb8f1-4ff9-4600-9695-8f92bb6e6300"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1914,19 +1927,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F143509-8442-4140-AEC8-97377484A183}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C8F6EB3-4135-4070-A5BE-B734AD9AC2FC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="612eb8f1-4ff9-4600-9695-8f92bb6e6300"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
TC 11 to 19
</commit_message>
<xml_diff>
--- a/BigID SGC Test Cases Document.xlsx
+++ b/BigID SGC Test Cases Document.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bluepineapple-my.sharepoint.com/personal/yuvraj_sonavane_bluepineapple_io/Documents/Documents/SGC_playwright/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{0716156C-7DEA-41C4-8C6E-FDBEBB68CB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{298C1D19-D869-4683-9ADE-40E155DF22D7}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{0716156C-7DEA-41C4-8C6E-FDBEBB68CB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{018253C7-06F5-4674-B49B-8803AE106F8A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test cases" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="140">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -398,9 +398,6 @@
 4. Click save &amp; validate button</t>
   </si>
   <si>
-    <t>Configuration should be saved even though the classification group is invalid</t>
-  </si>
-  <si>
     <t>1. Change classification group and/or batch size
 2. Click save and validate button
 3. Trigger the next scheduled import run</t>
@@ -417,9 +414,6 @@
     <t>Job logs Start and End, staging table should be  populated with the expected records for all eligible data sources and catalogs, no errors logged</t>
   </si>
   <si>
-    <t>Error should be logged in system logs</t>
-  </si>
-  <si>
     <t>Error should be logged in the system logs</t>
   </si>
   <si>
@@ -499,6 +493,15 @@
   </si>
   <si>
     <t>Leave export data sources empty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration should not be saved </t>
+  </si>
+  <si>
+    <t>Should not allow to run the import job to begin with</t>
+  </si>
+  <si>
+    <t>Error Not logged anywhere</t>
   </si>
 </sst>
 </file>
@@ -546,7 +549,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -568,6 +571,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE4E4"/>
+        <bgColor rgb="FFFCE4E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF7C80"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF7C80"/>
         <bgColor rgb="FFFCE4E4"/>
       </patternFill>
     </fill>
@@ -599,7 +614,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -628,12 +643,26 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF7C80"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1031,7 +1060,7 @@
         <v>25</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>29</v>
@@ -1060,7 +1089,7 @@
         <v>25</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>29</v>
@@ -1234,7 +1263,7 @@
         <v>34</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>27</v>
@@ -1275,7 +1304,7 @@
         <v>106</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>107</v>
@@ -1307,7 +1336,7 @@
         <v>46</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>109</v>
+        <v>137</v>
       </c>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
@@ -1330,13 +1359,13 @@
         <v>31</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>48</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
@@ -1359,13 +1388,13 @@
         <v>28</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>50</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
@@ -1394,39 +1423,39 @@
         <v>54</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
     </row>
     <row r="16" spans="1:11" ht="52" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="H16" s="11" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="39" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" ht="39" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>56</v>
       </c>
@@ -1443,16 +1472,19 @@
         <v>28</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="78" x14ac:dyDescent="0.35">
+        <v>113</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="78" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>57</v>
       </c>
@@ -1469,16 +1501,16 @@
         <v>28</v>
       </c>
       <c r="F18" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="H18" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="G18" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="65" x14ac:dyDescent="0.35">
+    </row>
+    <row r="19" spans="1:9" ht="65" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>58</v>
       </c>
@@ -1495,16 +1527,19 @@
         <v>28</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="52" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="52" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>59</v>
       </c>
@@ -1524,13 +1559,13 @@
         <v>76</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="52" x14ac:dyDescent="0.35">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="52" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>60</v>
       </c>
@@ -1547,16 +1582,16 @@
         <v>28</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="52" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="52" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>61</v>
       </c>
@@ -1576,13 +1611,13 @@
         <v>77</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="52" x14ac:dyDescent="0.35">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="52" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>62</v>
       </c>
@@ -1599,16 +1634,16 @@
         <v>28</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="52" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="52" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>63</v>
       </c>
@@ -1628,13 +1663,13 @@
         <v>79</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="52" x14ac:dyDescent="0.35">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="52" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>64</v>
       </c>
@@ -1654,10 +1689,10 @@
         <v>82</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="39" x14ac:dyDescent="0.35">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="39" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
         <v>65</v>
       </c>
@@ -1674,14 +1709,14 @@
         <v>28</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G26" s="7"/>
       <c r="H26" s="7" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="39" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="39" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>66</v>
       </c>
@@ -1698,14 +1733,14 @@
         <v>28</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G27" s="7"/>
       <c r="H27" s="7" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="39" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="39" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
         <v>67</v>
       </c>
@@ -1722,14 +1757,14 @@
         <v>28</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G28" s="7"/>
       <c r="H28" s="7" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="3"/>
     </row>
   </sheetData>
@@ -1740,6 +1775,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100404C0165E0195B418F91E482819B929E" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e4c9b75cb2d32282968581d314e0945">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="612eb8f1-4ff9-4600-9695-8f92bb6e6300" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="506a22593d787f6cb6aee14c493b0560" ns2:_="">
     <xsd:import namespace="612eb8f1-4ff9-4600-9695-8f92bb6e6300"/>
@@ -1877,35 +1927,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F143509-8442-4140-AEC8-97377484A183}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C8F6EB3-4135-4070-A5BE-B734AD9AC2FC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="612eb8f1-4ff9-4600-9695-8f92bb6e6300"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1927,9 +1952,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C8F6EB3-4135-4070-A5BE-B734AD9AC2FC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F143509-8442-4140-AEC8-97377484A183}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="612eb8f1-4ff9-4600-9695-8f92bb6e6300"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>